<commit_message>
Mise a jour automatique de la collection et de la page Wanted
</commit_message>
<xml_diff>
--- a/01_Liste achat.xlsx
+++ b/01_Liste achat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PHILIPPE\Desktop\Sauvegarde vinyles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCE8CDE-E68E-4422-BD00-A7BC3AEC993C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21FB8BAB-8C52-4BB3-A0CE-07B701451D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1229" uniqueCount="809">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1229" uniqueCount="810">
   <si>
     <t>Artistes / Titres</t>
   </si>
@@ -2470,6 +2470,9 @@
   </si>
   <si>
     <t>MASS PRODUCTION - Come And Get Some Of This</t>
+  </si>
+  <si>
+    <t>LUTHER VANDROSS - She's a super lady</t>
   </si>
 </sst>
 </file>
@@ -13158,7 +13161,7 @@
     </row>
     <row r="303" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
-        <v>279</v>
+        <v>809</v>
       </c>
       <c r="B303" s="21"/>
       <c r="C303" s="3"/>

</xml_diff>